<commit_message>
incorpora columna corredor a excel historial de cotizaciones
</commit_message>
<xml_diff>
--- a/Historial_cotizaciones.xlsx
+++ b/Historial_cotizaciones.xlsx
@@ -1,50 +1,113 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AI\cotizador-web-mp\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D171B221-34E3-495B-AAD5-D9BFBFA56756}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Historial" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="27">
+  <si>
+    <t>N° Cotización</t>
+  </si>
+  <si>
+    <t>Fecha</t>
+  </si>
+  <si>
+    <t>Proyecto</t>
+  </si>
+  <si>
+    <t>Comuna</t>
+  </si>
+  <si>
+    <t>N° Unidad</t>
+  </si>
+  <si>
+    <t>Tipo Unidad</t>
+  </si>
+  <si>
+    <t>Broker/Cliente</t>
+  </si>
+  <si>
+    <t>Valor Venta UF</t>
+  </si>
+  <si>
+    <t>Crédito Hip. UF</t>
+  </si>
+  <si>
+    <t>Pie %</t>
+  </si>
+  <si>
+    <t>COT-2026-0005</t>
+  </si>
+  <si>
+    <t>31 de marzo de 2026</t>
+  </si>
+  <si>
+    <t>ALTO BUZETA (MT)</t>
+  </si>
+  <si>
+    <t>Cerrillos</t>
+  </si>
+  <si>
+    <t>Departamento</t>
+  </si>
+  <si>
+    <t>Verónica Valdés</t>
+  </si>
+  <si>
+    <t>COT-2026-0004</t>
+  </si>
+  <si>
+    <t>Felipe Donoso</t>
+  </si>
+  <si>
+    <t>COT-2026-0003</t>
+  </si>
+  <si>
+    <t>JARDINES DE ALVARADO</t>
+  </si>
+  <si>
+    <t>Independencia</t>
+  </si>
+  <si>
+    <t>jp</t>
+  </si>
+  <si>
+    <t>COT-2026-0002</t>
+  </si>
+  <si>
+    <t>felipe donoso</t>
+  </si>
+  <si>
+    <t>COT-2026-0001</t>
+  </si>
+  <si>
+    <t>juan perez</t>
+  </si>
+  <si>
+    <t>Corredor</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="10">
-    <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0;[Red]&quot;$&quot;\-#,##0"/>
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="165" formatCode="[$$]#,##0"/>
-    <numFmt numFmtId="166" formatCode="[$UF]#,##0.0"/>
-    <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.0"/>
-    <numFmt numFmtId="168" formatCode="[$UF]#,##0.00"/>
-    <numFmt numFmtId="169" formatCode="0.000000%"/>
-    <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -74,13 +137,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4">
+    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{6392AFE7-D39C-4622-AC8C-E6765621BD07}"/>
+  </tableStyles>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -405,74 +478,77 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J6"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:K6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="25.83203125" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" customWidth="1"/>
-    <col min="9" max="9" width="15.83203125" customWidth="1"/>
-    <col min="10" max="10" width="8.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.796875" customWidth="1"/>
+    <col min="2" max="2" width="14.796875" customWidth="1"/>
+    <col min="3" max="3" width="30.796875" customWidth="1"/>
+    <col min="4" max="4" width="16.796875" customWidth="1"/>
+    <col min="5" max="5" width="10.796875" customWidth="1"/>
+    <col min="6" max="6" width="14.796875" customWidth="1"/>
+    <col min="7" max="7" width="25.796875" customWidth="1"/>
+    <col min="8" max="9" width="15.796875" customWidth="1"/>
+    <col min="10" max="10" width="8.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>N° Cotización</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Fecha</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Proyecto</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Comuna</v>
-      </c>
-      <c r="E1" t="str">
-        <v>N° Unidad</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Tipo Unidad</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Broker/Cliente</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Valor Venta UF</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Crédito Hip. UF</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Pie %</v>
+    <row r="1" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>26</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>COT-2026-0005</v>
-      </c>
-      <c r="B2" t="str">
-        <v>31 de marzo de 2026</v>
-      </c>
-      <c r="C2" t="str">
-        <v>ALTO BUZETA (MT)</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Cerrillos</v>
+    <row r="2" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
+        <v>13</v>
       </c>
       <c r="E2">
         <v>1813</v>
       </c>
-      <c r="F2" t="str">
-        <v>Departamento</v>
-      </c>
-      <c r="G2" t="str">
-        <v>Verónica Valdés</v>
+      <c r="F2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" t="s">
+        <v>15</v>
       </c>
       <c r="H2">
         <v>3328.3</v>
@@ -484,27 +560,27 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>COT-2026-0004</v>
-      </c>
-      <c r="B3" t="str">
-        <v>31 de marzo de 2026</v>
-      </c>
-      <c r="C3" t="str">
-        <v>ALTO BUZETA (MT)</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Cerrillos</v>
+    <row r="3" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
       </c>
       <c r="E3">
         <v>813</v>
       </c>
-      <c r="F3" t="str">
-        <v>Departamento</v>
-      </c>
-      <c r="G3" t="str">
-        <v>Felipe Donoso</v>
+      <c r="F3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" t="s">
+        <v>17</v>
       </c>
       <c r="H3">
         <v>2802.6</v>
@@ -516,27 +592,27 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>COT-2026-0003</v>
-      </c>
-      <c r="B4" t="str">
-        <v>31 de marzo de 2026</v>
-      </c>
-      <c r="C4" t="str">
-        <v>JARDINES DE ALVARADO</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Independencia</v>
+    <row r="4" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" t="s">
+        <v>20</v>
       </c>
       <c r="E4">
         <v>217</v>
       </c>
-      <c r="F4" t="str">
-        <v>Departamento</v>
-      </c>
-      <c r="G4" t="str">
-        <v>jp</v>
+      <c r="F4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" t="s">
+        <v>21</v>
       </c>
       <c r="H4">
         <v>2349.87</v>
@@ -548,27 +624,27 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>COT-2026-0002</v>
-      </c>
-      <c r="B5" t="str">
-        <v>31 de marzo de 2026</v>
-      </c>
-      <c r="C5" t="str">
-        <v>ALTO BUZETA (MT)</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Cerrillos</v>
+    <row r="5" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" t="s">
+        <v>13</v>
       </c>
       <c r="E5">
         <v>809</v>
       </c>
-      <c r="F5" t="str">
-        <v>Departamento</v>
-      </c>
-      <c r="G5" t="str">
-        <v>felipe donoso</v>
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" t="s">
+        <v>23</v>
       </c>
       <c r="H5">
         <v>2781</v>
@@ -580,27 +656,27 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>COT-2026-0001</v>
-      </c>
-      <c r="B6" t="str">
-        <v>31 de marzo de 2026</v>
-      </c>
-      <c r="C6" t="str">
-        <v>ALTO BUZETA (MT)</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Cerrillos</v>
+    <row r="6" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" t="s">
+        <v>13</v>
       </c>
       <c r="E6">
         <v>808</v>
       </c>
-      <c r="F6" t="str">
-        <v>Departamento</v>
-      </c>
-      <c r="G6" t="str">
-        <v>juan perez</v>
+      <c r="F6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" t="s">
+        <v>25</v>
       </c>
       <c r="H6">
         <v>2781</v>
@@ -613,8 +689,9 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J6"/>
+    <ignoredError sqref="A1:J6" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix llenado historial cotizaciones
</commit_message>
<xml_diff>
--- a/Historial_cotizaciones.xlsx
+++ b/Historial_cotizaciones.xlsx
@@ -1,26 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AI\cotizador-web-mp\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D171B221-34E3-495B-AAD5-D9BFBFA56756}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Historial" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Historial" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>N° Cotización</t>
   </si>
@@ -52,68 +43,41 @@
     <t>Pie %</t>
   </si>
   <si>
-    <t>COT-2026-0005</t>
-  </si>
-  <si>
-    <t>31 de marzo de 2026</t>
-  </si>
-  <si>
-    <t>ALTO BUZETA (MT)</t>
-  </si>
-  <si>
-    <t>Cerrillos</t>
+    <t>Corredor</t>
+  </si>
+  <si>
+    <t>TEST-0001</t>
+  </si>
+  <si>
+    <t>10-04-2026</t>
+  </si>
+  <si>
+    <t>PROYECTO TEST</t>
+  </si>
+  <si>
+    <t>Santiago</t>
   </si>
   <si>
     <t>Departamento</t>
   </si>
   <si>
-    <t>Verónica Valdés</t>
-  </si>
-  <si>
-    <t>COT-2026-0004</t>
-  </si>
-  <si>
-    <t>Felipe Donoso</t>
-  </si>
-  <si>
-    <t>COT-2026-0003</t>
-  </si>
-  <si>
-    <t>JARDINES DE ALVARADO</t>
-  </si>
-  <si>
-    <t>Independencia</t>
-  </si>
-  <si>
-    <t>jp</t>
-  </si>
-  <si>
-    <t>COT-2026-0002</t>
-  </si>
-  <si>
-    <t>felipe donoso</t>
-  </si>
-  <si>
-    <t>COT-2026-0001</t>
-  </si>
-  <si>
-    <t>juan perez</t>
-  </si>
-  <si>
-    <t>Corredor</t>
+    <t>Juan Test</t>
+  </si>
+  <si>
+    <t>Corredor Test</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -143,9 +107,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4">
-    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{6392AFE7-D39C-4622-AC8C-E6765621BD07}"/>
-  </tableStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -478,22 +440,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="18.796875" customWidth="1"/>
-    <col min="2" max="2" width="14.796875" customWidth="1"/>
-    <col min="3" max="3" width="30.796875" customWidth="1"/>
-    <col min="4" max="4" width="16.796875" customWidth="1"/>
-    <col min="5" max="5" width="10.796875" customWidth="1"/>
-    <col min="6" max="6" width="14.796875" customWidth="1"/>
-    <col min="7" max="7" width="25.796875" customWidth="1"/>
-    <col min="8" max="9" width="15.796875" customWidth="1"/>
-    <col min="10" max="10" width="8.796875" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -525,173 +476,46 @@
         <v>9</v>
       </c>
       <c r="K1" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E2">
-        <v>1813</v>
+        <v>101</v>
       </c>
       <c r="F2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H2">
-        <v>3328.3</v>
+        <v>2800</v>
       </c>
       <c r="I2">
-        <v>3161.89</v>
+        <v>2500</v>
       </c>
       <c r="J2">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3">
-        <v>813</v>
-      </c>
-      <c r="F3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G3" t="s">
+      <c r="K2" t="s">
         <v>17</v>
-      </c>
-      <c r="H3">
-        <v>2802.6</v>
-      </c>
-      <c r="I3">
-        <v>2522.34</v>
-      </c>
-      <c r="J3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E4">
-        <v>217</v>
-      </c>
-      <c r="F4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G4" t="s">
-        <v>21</v>
-      </c>
-      <c r="H4">
-        <v>2349.87</v>
-      </c>
-      <c r="I4">
-        <v>2114.88</v>
-      </c>
-      <c r="J4">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5">
-        <v>809</v>
-      </c>
-      <c r="F5" t="s">
-        <v>14</v>
-      </c>
-      <c r="G5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H5">
-        <v>2781</v>
-      </c>
-      <c r="I5">
-        <v>2641.95</v>
-      </c>
-      <c r="J5">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" t="s">
-        <v>13</v>
-      </c>
-      <c r="E6">
-        <v>808</v>
-      </c>
-      <c r="F6" t="s">
-        <v>14</v>
-      </c>
-      <c r="G6" t="s">
-        <v>25</v>
-      </c>
-      <c r="H6">
-        <v>2781</v>
-      </c>
-      <c r="I6">
-        <v>2502.9</v>
-      </c>
-      <c r="J6">
-        <v>10</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:J6" numberStoredAsText="1"/>
-  </ignoredErrors>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>